<commit_message>
Verify stage 1 table against manufacturer data; add stage 5 inputs
- GT 63 4-Door Coupé checked against the Mercedes-Benz Media press kit:
  kerb weight 2460 kg (DIN), WLTP 17.9-21.0 kWh/100 km, 0-100 in 2.4 s
  (2.1 s with 1-foot rollout), continuous power 530 kW; GT 55 figures
- Filled official Cx / mass / consumption / transmission for Porsche,
  Audi, Lotus, Lucid and Rimac; corrected Lucid (908 kW, 1940 Nm),
  Rimac (2340 Nm) and Lotus (705 V nominal, 2-speed rear only on
  900 Sport Carbon)
- Added source URLs for every changed value; Tesla, Maserati and
  Xiaomi stay partly secondary (sites block automated access)
- README: updated summary table and new "Date pentru etapa 5" section

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dz8sSyt3zaur1x4jsnU1sR
</commit_message>
<xml_diff>
--- a/etapa1-documentare/CCA_Etapa1_Documentare.xlsx
+++ b/etapa1-documentare/CCA_Etapa1_Documentare.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Tabel comparativ" sheetId="1" state="visible" r:id="rId3"/>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="257">
   <si>
     <t xml:space="preserve">Etapa 1 – Documentare: acționări electrice pe automobile electrice de înaltă performanță (GT / super-sport)</t>
   </si>
@@ -158,7 +158,7 @@
     <t xml:space="preserve">3 motoare sincrone cu flux axial (YASA): 2 pe puntea spate + 1 pe puntea față, integrate în 2 unități HP.EDU (motor + reductor + invertor)</t>
   </si>
   <si>
-    <t xml:space="preserve">Spate: câte un reductor planetar pentru fiecare motor; față: reductor cu roți dințate cilindrice</t>
+    <t xml:space="preserve">Spate: câte un set planetar compact pentru fiecare motor (o carcasă comună); față: reductor cu roți dințate cilindrice + unitate de decuplare (DCU)</t>
   </si>
   <si>
     <t xml:space="preserve">≈114</t>
@@ -170,7 +170,7 @@
     <t xml:space="preserve">O / S</t>
   </si>
   <si>
-    <t xml:space="preserve">Valori declarate pentru concept (simulări / prototipuri): v_max &gt;360 km/h, P &gt;1000 kW, încărcare DC &gt;850 kW. Record Nardò 08/2025: 40 075 km în 7 zile 13 h 24 min. Capacitatea bateriei (≈114 kWh) provine din presă.</t>
+    <t xml:space="preserve">Valori declarate pentru concept: v_max &gt;360 km/h, P &gt;1000 kW, încărcare DC &gt;850 kW (medie), Cx 0,198, arie frontală 2,24 m², &gt;3000 celule cilindrice NCMA. Record Nardò 08/2025: 5479 km în 24 h; 40 075 km în 7 zile 13 h 24 min. Mercedes nu publică capacitatea bateriei și cuplul conceptului – ≈114 kWh provine din presă (S).</t>
   </si>
   <si>
     <t xml:space="preserve">GT 63 4MATIC+ 4-Door Coupé (AMG.EA)</t>
@@ -179,22 +179,22 @@
     <t xml:space="preserve">Serie (prezentat 05/2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">3 motoare sincrone cu flux axial (fabricate la Berlin-Marienfelde): 2 spate + 1 față, în unități HP.EDU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spate: câte un reductor planetar de intrare pentru fiecare motor (o singură carcasă)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">106 (util)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈2460–2535</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Versiunea de serie derivată din GT XX. 860 kW = putere de vârf cu AMG Launch Control; v_max 300 km/h cu Driver's Package; 2660 celule cilindrice răcite direct în ulei; încărcare DC 600 kW. Varianta GT 55: 600 kW, autonomie WLTP 700 km. Masa și consumul diferă între surse (2460 / 2535 kg; 17,9 / 18,2 kWh/100 km).</t>
+    <t xml:space="preserve">3 motoare sincrone cu flux axial (YASA, fabricate la Berlin-Marienfelde): 2 spate + 1 față, în unități HP.EDU; 3 invertoare SiC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spate: reductor planetar cu o treaptă, carcasă comună pentru cele 2 motoare; față: reductor cu roți dințate cilindrice + unitate de decuplare (DCU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">106 (net)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17,9–21,0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">860 kW = putere de vârf cu AMG Launch Control la 80 % SoC; putere continuă 530 kW; boost 63 s. 0–100 km/h: 2,4 s (2,1 s cu „1-foot rollout”); 0–200 km/h: 6,8 s (6,4 s). v_max 300 km/h cu Driver's Package. Masa = DIN (fără șofer); ≈2535 kg în varianta UE cu șofer de 75 kg. Arie frontală 2,44 m². 2660 celule cilindrice NCMA răcite direct în ulei; DC 600 kW. WLTP 596–696 km. GT 55: 600 kW (continuu 375 kW), 1800 Nm, 2,8 s (2,5 s rollout), 2460 kg, 17,8–21,0 kWh/100 km, WLTP 597–700 km.</t>
   </si>
   <si>
     <t xml:space="preserve">Porsche</t>
@@ -215,13 +215,10 @@
     <t xml:space="preserve">97 net / 105 brut</t>
   </si>
   <si>
-    <t xml:space="preserve">20,5–21,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">580 kW putere maximă; 760 kW overboost cu Launch Control (815 kW timp de 2 s); Attack Mode +120 kW / 10 s. Consumul WLTP este cel publicat pentru Taycan Turbo GT.</t>
+    <t xml:space="preserve">20,6–21,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">580 kW putere maximă; 760 kW overboost cu Launch Control (815 kW timp de 2 s); Attack Mode +120 kW / 10 s. Date pentru pachetul Weissach (fișa tehnică UE 03/2024): masă DIN, arie frontală 2,35 m², anvelope 265/35 ZR21 / 305/30 ZR21.</t>
   </si>
   <si>
     <t xml:space="preserve">Audi</t>
@@ -236,7 +233,7 @@
     <t xml:space="preserve">18,7–20,8</t>
   </si>
   <si>
-    <t xml:space="preserve">550 kW nominal / 680 kW cu Launch Control; push-to-pass +70 kW / 10 s. Putere continuă declarată: 163 kW – singurul producător din tabel care o publică (date nominale).</t>
+    <t xml:space="preserve">550 kW nominal / 680 kW cu Launch Control; push-to-pass +70 kW / 10 s. Cuplu motoare față / spate: 409 / 590 Nm. Putere continuă declarată: 163 kW. Masa = fără șofer (2395 kg cu șofer); arie frontală 2,35 m².</t>
   </si>
   <si>
     <t xml:space="preserve">Lotus</t>
@@ -248,45 +245,48 @@
     <t xml:space="preserve">2 motoare electrice: 1 față + 1 spate (tracțiune integrală)</t>
   </si>
   <si>
-    <t xml:space="preserve">Spate: cutie cu 2 trepte (de verificat)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈18,7</t>
+    <t xml:space="preserve">Față: o treaptă; spate: cutie cu 2 trepte (doar la versiunea 900 Sport Carbon; 900 Sport are o treaptă și spate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">102 (brut)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">705 (nominal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17,7–22,4 (gama Emeya)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Putere, cuplu, v_max, 0–100, baterie, tensiune nominală (705 V; „arhitectură 800 V” în marketing), transmisie și autonomia WLTP 435–485 km sunt din fișa de presă Lotus. Masa (S) nu este publicată de Lotus; consumul oficial este dat doar pentru toată gama.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tesla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model S Plaid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serie (2021)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 motoare sincrone cu magneți permanenți: 1 față + 2 spate (câte unul pe roată)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reductor cu o treaptă pentru fiecare unitate de acționare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≈96 (util)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≈400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≈15,7</t>
   </si>
   <si>
     <t xml:space="preserve">S</t>
   </si>
   <si>
-    <t xml:space="preserve">Încărcare DC 400 kW; autonomie WLTP ≈535 km.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tesla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model S Plaid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serie (2021)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 motoare sincrone cu magneți permanenți: 1 față + 2 spate (câte unul pe roată)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reductor cu o treaptă pentru fiecare unitate de acționare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈96 (util)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈15,7</t>
-  </si>
-  <si>
     <t xml:space="preserve">322 km/h cu Track Package; arhitectură de 400 V (singura din tabel); încărcare DC 250 kW; autonomie WLTP ≈611 km.</t>
   </si>
   <si>
@@ -305,6 +305,9 @@
     <t xml:space="preserve">3 motoare sincrone cu magneți permanenți: 1 față + 2 spate</t>
   </si>
   <si>
+    <t xml:space="preserve">O treaptă: raport 7:1 (față), 6,8:1 (spate)</t>
+  </si>
+  <si>
     <t xml:space="preserve">118</t>
   </si>
   <si>
@@ -314,7 +317,7 @@
     <t xml:space="preserve">≈17,2 (EPA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Putere declarată 1234 CP (≈920 kW); cuplu 1430 lb-ft (≈1939 Nm); masă 5336 lb. Consumul este calculat din eficiența EPA de 3,61 mi/kWh (nu WLTP).</t>
+    <t xml:space="preserve">Fișa tehnică 2024: 1234 hp (908 kW), 1430 lb-ft (1940 Nm), v_max 205 mph, masă 5336 lb. Anvelope 265/35R20 / 295/30R21. Consumul este calculat din eficiența EPA de 3,61 mi/kWh (nu WLTP).</t>
   </si>
   <si>
     <t xml:space="preserve">Xiaomi</t>
@@ -329,10 +332,16 @@
     <t xml:space="preserve">3 motoare: 2 × HyperEngine V8s (425 kW, 635 Nm, 27 200 rpm) + 1 × V6s (288 kW)</t>
   </si>
   <si>
+    <t xml:space="preserve">Reductor cu o treaptă pentru fiecare motor</t>
+  </si>
+  <si>
     <t xml:space="preserve">93,7 net / 95 brut</t>
   </si>
   <si>
-    <t xml:space="preserve">Baterie CATL Qilin 2.0 (putere maximă de descărcare 1330 kW).</t>
+    <t xml:space="preserve">≈16,5 (CLTC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baterie CATL Qilin 2.0 (putere maximă de descărcare 1330 kW). Consumul este pe ciclul chinezesc CLTC (nu WLTP); Cx-ul versiunii Ultra (cu eleron) nu este publicat (0,195 este valoarea SU7 standard).</t>
   </si>
   <si>
     <t xml:space="preserve">BYD (Yangwang)</t>
@@ -347,7 +356,7 @@
     <t xml:space="preserve">80 (LFP Blade)</t>
   </si>
   <si>
-    <t xml:space="preserve">v_max = 309,19 km/h. Varianta U9 Track Edition / Xtreme: 1200 V, &gt;2200 kW, 496,22 km/h (09/2025, record într-un singur sens).</t>
+    <t xml:space="preserve">Comunicat BYD: ≈1300 CP, 1680 Nm, 309,19 km/h, 0–100 km/h 2,36 s, 4 motoare independente (O); masa, tensiunea și bateria sunt din surse secundare. Varianta U9 Track Edition / Xtreme: 1200 V, &gt;2200 kW, 496,22 km/h (09/2025, record într-un singur sens).</t>
   </si>
   <si>
     <t xml:space="preserve">Rimac</t>
@@ -362,7 +371,7 @@
     <t xml:space="preserve">4 motoare sincrone cu magneți permanenți (rotor cu manșon din carbon): față 2 × 220 kW / 280 Nm, spate 2 × 480 kW / 900 Nm; 4 invertoare</t>
   </si>
   <si>
-    <t xml:space="preserve">4 reductoare independente (câte unul pe motor)</t>
+    <t xml:space="preserve">Față: 2 reductoare cu o treaptă (la capetele punții); spate: reductor dublu cu o treaptă (2 reductoare într-o carcasă)</t>
   </si>
   <si>
     <t xml:space="preserve">120</t>
@@ -371,7 +380,10 @@
     <t xml:space="preserve">730 (max.)</t>
   </si>
   <si>
-    <t xml:space="preserve">6960 celule cilindrice 21700; încărcare DC 500 kW; autonomie ≈490 km. Cuplul la roată declarat: 13 430 Nm.</t>
+    <t xml:space="preserve">30,0 (WLTP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6960 celule cilindrice 21700; încărcare DC 500 kW; autonomie WLTP 490 km. Cuplu la motoare 2340 Nm, la roți 13 430 Nm. 0–100 km/h cu „1-foot rollout”. Cx 0,30 în modul low-drag. Pagina web Rimac indică 226 / 450 kW pe motor (fișa PDF: 220 / 480 kW).</t>
   </si>
   <si>
     <t xml:space="preserve">Maserati</t>
@@ -386,10 +398,7 @@
     <t xml:space="preserve">83 net / 92,5 brut</t>
   </si>
   <si>
-    <t xml:space="preserve">≈2335</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Putere limitată de baterie la 560 kW (≈610 kW în regim de boost, sursă secundară). Masa = 5148 lb (UE, neîncărcat).</t>
+    <t xml:space="preserve">Putere limitată de baterie la 560 kW (≈610 kW în regim de boost, sursă secundară). Masa 2260 kg = „masă omologată” din comunicatul Stellantis (citit doar prin motorul de căutare; site-urile Maserati / Stellantis blochează accesul automat). Cx raportat diferit (0,26 / 0,27) – nepreluat.</t>
   </si>
   <si>
     <t xml:space="preserve">Factor conversie kW → CP (cal-putere metric):</t>
@@ -527,10 +536,10 @@
     <t xml:space="preserve">Ședința 14 rămâne rezervă (recuperări / susțineri restante).</t>
   </si>
   <si>
-    <t xml:space="preserve">Surse (accesate 07.10.2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notă: paginile au fost consultate prin motor de căutare; valorile marcate S trebuie verificate pe pagina producătorului înainte de predare. Datele de concept nu sunt valori omologate.</t>
+    <t xml:space="preserve">Surse (accesate 07.10.2026; verificare directă a paginilor producătorilor la 07.10.2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notă: Mercedes, Porsche, Audi, Lotus, Lucid, Rimac și BYD au fost verificate direct pe documentele producătorului. Tesla, Maserati și Xiaomi blochează accesul automat – valorile lor rămân parțial S. Datele de concept nu sunt valori omologate.</t>
   </si>
   <si>
     <t xml:space="preserve">Vehicul</t>
@@ -581,9 +590,45 @@
     <t xml:space="preserve">https://www.drivencarguide.co.nz/news/mercedes-amgs-concept-amg-gt-xx-packs-serious-tech-under-throwback-looks/</t>
   </si>
   <si>
+    <t xml:space="preserve">Mercedes-Benz Media – comunicat CONCEPT AMG GT XX (date tehnice, Cx, arie frontală)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://media.mercedes-benz.com/en/article/dc62bb92-5082-42f1-bc9a-c838bc09e985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mercedes-Benz Media – recorduri Nardò 08/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://media.mercedes-benz.com/en/article/b2d73049-f14b-4019-8da3-a0dd5e6dfb89</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mercedes-AMG GT 63 4-Door Coupé</t>
   </si>
   <si>
+    <t xml:space="preserve">Mercedes-Benz Media – comunicat de lansare 20.05.2026 (tabele tehnice GT 63 / GT 55)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://media.mercedes-benz.com/en/article/c8b7109f-2287-4070-b776-9204da1513ef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mercedes-Benz Media – start comenzi 27.05.2026 (consum WLTP, nota „1-foot rollout”)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://media.mercedes-benz.com/article/f037de81-64ba-4236-b555-75a5f4c3a56b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mercedes-Benz Media – motorul cu flux axial, HP.EDU cu reductor planetar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://media.mercedes-benz.com/en/article/bebac2af-acdc-465a-9538-adb0bf3d8ccf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mercedes-Benz Media – GT 53 4-Door Coupé (aceeași caroserie: arie frontală 2,44 m²)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://media.mercedes-benz.com/en/article/0955928c-b613-41b4-b754-08399bbfcccc</t>
+  </si>
+  <si>
     <t xml:space="preserve">mercedes-amg.com – GT 4-Door Coupé</t>
   </si>
   <si>
@@ -665,45 +710,69 @@
     <t xml:space="preserve">Lotus Emeya R</t>
   </si>
   <si>
+    <t xml:space="preserve">Lotus – presă, specificații tehnice Emeya (putere, cuplu, transmisie, 705 V, WLTP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lotuscars.com/en/press/models/emeya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lotus – pagina de specificații Emeya (consum WLTP gamă, „2 speed trans.”)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lotuscars.com/en-GB/emeya/specifications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">evkx.net – fișă tehnică (masă)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://evkx.net/models/lotus/emeya/emeya_r/specifications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CarNewsChina – baza de date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://data.carnewschina.com/database/lotus/lotus-emeya/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tesla Model S Plaid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">evkx.net – fișă tehnică (inclusiv Cx 0,208)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://evkx.net/models/tesla/model_s/model_s_plaid/specifications/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucid Air Sapphire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucid – specificații finale de producție</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://lucidmotors.com/stories/final-production-specs-sapphire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucid – fișă tehnică 2024 (PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://lucidmotors.com/media/document/lucid-air-sapphire-technical-specs-2024.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xiaomi SU7 Ultra</t>
+  </si>
+  <si>
     <t xml:space="preserve">evkx.net – fișă tehnică</t>
   </si>
   <si>
-    <t xml:space="preserve">https://evkx.net/models/lotus/emeya/emeya_r/specifications</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CarNewsChina – baza de date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://data.carnewschina.com/database/lotus/lotus-emeya/2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tesla Model S Plaid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://evkx.net/models/tesla/model_s/model_s_plaid/specifications/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lucid Air Sapphire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lucid – specificații finale de producție</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://lucidmotors.com/stories/final-production-specs-sapphire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lucid – fișă tehnică 2024 (PDF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://lucidmotors.com/media/document/lucid-air-sapphire-technical-specs-2024.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xiaomi SU7 Ultra</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://evkx.net/models/xiaomi/su7/su7_ultra/specifications</t>
   </si>
   <si>
+    <t xml:space="preserve">ZOL – parametri SU7 Ultra (consum CLTC 16,5 kWh/100 km)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://detail.zol.com.cn/2113/2112093/param.shtml</t>
+  </si>
+  <si>
     <t xml:space="preserve">CarNewsChina – lansare SU7 Ultra / V8s</t>
   </si>
   <si>
@@ -713,6 +782,12 @@
     <t xml:space="preserve">Yangwang U9</t>
   </si>
   <si>
+    <t xml:space="preserve">BYD – comunicat de lansare U9 (1680 Nm, 309,19 km/h, 2,36 s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.byd.com/us/news-list/YANGWANG-Launched-the-U9-Priced-at-1-68-Million-RMB</t>
+  </si>
+  <si>
     <t xml:space="preserve">autotijd.be – fișă tehnică</t>
   </si>
   <si>
@@ -737,10 +812,10 @@
     <t xml:space="preserve">Rimac – specificații tehnice (PDF)</t>
   </si>
   <si>
-    <t xml:space="preserve">https://web-cdn.rimac-automobili.com/wp-content/uploads/2023/11/20171226/Nevera_Technical-specifications.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rimac – Nevera</t>
+    <t xml:space="preserve">https://cloudfront.rimac-automobili.com/wp-content/uploads/2023/11/20171226/Nevera_Technical-specifications.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rimac – Nevera (consum WLTP 30,0 kWh/100 km, Cx 0,3)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.rimac-automobili.com/nevera/</t>
@@ -753,6 +828,12 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.maserati.com/us/en/models/granturismo/granturismo-folgore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stellantis Media – comunicat New Maserati GranTurismo (masă omologată 2260 kg; acces blocat, citit prin motor de căutare)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.media.stellantis.com/em-en/maserati/press/new-maserati-granturismo</t>
   </si>
   <si>
     <t xml:space="preserve">ArenaEV – fișă tehnică</t>
@@ -1455,7 +1536,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="n">
         <v>1</v>
       </c>
@@ -1512,7 +1593,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="n">
         <v>2</v>
       </c>
@@ -1539,7 +1620,7 @@
         <v>2000</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>33</v>
@@ -1553,23 +1634,23 @@
       <c r="M7" s="6" t="n">
         <v>800</v>
       </c>
-      <c r="N7" s="6" t="s">
+      <c r="N7" s="6" t="n">
+        <v>2460</v>
+      </c>
+      <c r="O7" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>37</v>
       </c>
       <c r="P7" s="10" t="n">
         <v>0.22</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="n">
         <v>3</v>
       </c>
@@ -1616,14 +1697,14 @@
       <c r="O8" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="P8" s="19" t="s">
-        <v>24</v>
+      <c r="P8" s="19" t="n">
+        <v>0.31</v>
       </c>
       <c r="Q8" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="R8" s="15" t="s">
         <v>46</v>
-      </c>
-      <c r="R8" s="15" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1631,10 +1712,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>48</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>49</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>41</v>
@@ -1656,7 +1737,7 @@
         <v>2.5</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K9" s="15" t="s">
         <v>43</v>
@@ -1667,31 +1748,31 @@
       <c r="M9" s="15" t="n">
         <v>800</v>
       </c>
-      <c r="N9" s="15" t="s">
-        <v>24</v>
+      <c r="N9" s="15" t="n">
+        <v>2320</v>
       </c>
       <c r="O9" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="P9" s="19" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="Q9" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="R9" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="P9" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q9" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="R9" s="15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="n">
         <v>5</v>
       </c>
       <c r="B10" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>53</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>54</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>41</v>
@@ -1713,16 +1794,16 @@
         <v>2.78</v>
       </c>
       <c r="J10" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="K10" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="K10" s="15" t="s">
+      <c r="L10" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="L10" s="15" t="s">
+      <c r="M10" s="15" t="s">
         <v>57</v>
-      </c>
-      <c r="M10" s="15" t="n">
-        <v>800</v>
       </c>
       <c r="N10" s="15" t="n">
         <v>2565</v>
@@ -1734,10 +1815,10 @@
         <v>24</v>
       </c>
       <c r="Q10" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="R10" s="15" t="s">
         <v>59</v>
-      </c>
-      <c r="R10" s="15" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1745,13 +1826,13 @@
         <v>6</v>
       </c>
       <c r="B11" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="D11" s="15" t="s">
         <v>62</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>63</v>
       </c>
       <c r="E11" s="15" t="n">
         <v>322</v>
@@ -1770,28 +1851,28 @@
         <v>2.1</v>
       </c>
       <c r="J11" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="K11" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="K11" s="15" t="s">
+      <c r="L11" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="L11" s="15" t="s">
+      <c r="M11" s="15" t="s">
         <v>66</v>
-      </c>
-      <c r="M11" s="15" t="s">
-        <v>67</v>
       </c>
       <c r="N11" s="15" t="n">
         <v>2178</v>
       </c>
       <c r="O11" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="P11" s="19" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="Q11" s="15" t="s">
         <v>68</v>
-      </c>
-      <c r="P11" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q11" s="15" t="s">
-        <v>59</v>
       </c>
       <c r="R11" s="15" t="s">
         <v>69</v>
@@ -1814,14 +1895,14 @@
         <v>330</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>920</v>
+        <v>908</v>
       </c>
       <c r="G12" s="17" t="n">
         <f aca="false">ROUND(F12*$C$19,0)</f>
-        <v>1251</v>
+        <v>1235</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>1939</v>
+        <v>1940</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>73</v>
@@ -1830,42 +1911,42 @@
         <v>74</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="L12" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="M12" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N12" s="15" t="n">
         <v>2420</v>
       </c>
       <c r="O12" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="P12" s="19" t="s">
         <v>24</v>
       </c>
       <c r="Q12" s="15" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="R12" s="15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="n">
         <v>8</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>350</v>
@@ -1884,13 +1965,13 @@
         <v>1.98</v>
       </c>
       <c r="J13" s="15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K13" s="15" t="s">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="L13" s="15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M13" s="15" t="n">
         <v>897</v>
@@ -1899,27 +1980,27 @@
         <v>2360</v>
       </c>
       <c r="O13" s="15" t="s">
-        <v>24</v>
+        <v>86</v>
       </c>
       <c r="P13" s="19" t="s">
         <v>24</v>
       </c>
       <c r="Q13" s="15" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="R13" s="15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="n">
         <v>9</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>41</v>
@@ -1941,13 +2022,13 @@
         <v>2.36</v>
       </c>
       <c r="J14" s="15" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K14" s="15" t="s">
         <v>24</v>
       </c>
       <c r="L14" s="15" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="M14" s="15" t="n">
         <v>800</v>
@@ -1962,24 +2043,24 @@
         <v>24</v>
       </c>
       <c r="Q14" s="15" t="s">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="R14" s="15" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="n">
         <v>10</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E15" s="15" t="n">
         <v>412</v>
@@ -1992,48 +2073,48 @@
         <v>1914</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>2360</v>
+        <v>2340</v>
       </c>
       <c r="I15" s="18" t="n">
         <v>1.81</v>
       </c>
       <c r="J15" s="15" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="K15" s="15" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="L15" s="15" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="M15" s="15" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="N15" s="15" t="n">
         <v>2300</v>
       </c>
       <c r="O15" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="P15" s="19" t="s">
-        <v>24</v>
+        <v>100</v>
+      </c>
+      <c r="P15" s="19" t="n">
+        <v>0.3</v>
       </c>
       <c r="Q15" s="15" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="R15" s="15" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="n">
         <v>11</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>72</v>
@@ -2055,19 +2136,19 @@
         <v>2.7</v>
       </c>
       <c r="J16" s="15" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="K16" s="15" t="s">
         <v>24</v>
       </c>
       <c r="L16" s="15" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="M16" s="15" t="n">
         <v>800</v>
       </c>
-      <c r="N16" s="15" t="s">
-        <v>102</v>
+      <c r="N16" s="15" t="n">
+        <v>2260</v>
       </c>
       <c r="O16" s="15" t="s">
         <v>24</v>
@@ -2079,33 +2160,33 @@
         <v>29</v>
       </c>
       <c r="R16" s="15" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="20" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C19" s="21" t="n">
         <v>1.35962</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="20" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E22" s="22" t="n">
         <f aca="false">SUMPRODUCT(1/COUNTIF(B6:B16,B6:B16))</f>
@@ -2114,16 +2195,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E23" s="23" t="n">
         <f aca="false">AVERAGE(F7:F16)</f>
-        <v>872.1</v>
+        <v>870.9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E24" s="23" t="n">
         <f aca="false">MAX(F7:F16)</f>
@@ -2132,7 +2213,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E25" s="22" t="n">
         <f aca="false">AVERAGE(E7:E16)</f>
@@ -2141,20 +2222,20 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E26" s="23" t="n">
         <f aca="false">AVERAGE(H7:H16)</f>
-        <v>1577.1</v>
+        <v>1575.2</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E27" s="22" t="n">
         <f aca="false">COUNTIF(M7:M16,"&gt;=800")+COUNTIF(M7:M16,"900+")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2187,12 +2268,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -2219,19 +2300,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>1</v>
@@ -2278,7 +2359,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G5" s="25" t="n">
         <f aca="false">DATE(2026,10,7)</f>
@@ -2342,7 +2423,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -2355,7 +2436,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="G6" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D6,G$4&lt;=$E6),1,0)</f>
@@ -2419,7 +2500,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>2</v>
@@ -2433,7 +2514,7 @@
         <v>3</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G7" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D7,G$4&lt;=$E7),1,0)</f>
@@ -2497,7 +2578,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>2</v>
@@ -2511,7 +2592,7 @@
         <v>3</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G8" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D8,G$4&lt;=$E8),1,0)</f>
@@ -2573,7 +2654,7 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30"/>
       <c r="B9" s="31" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C9" s="30" t="n">
         <v>0</v>
@@ -2587,7 +2668,7 @@
         <v>3</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G9" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D9,G$4&lt;=$E9),1,0)</f>
@@ -2651,7 +2732,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>2</v>
@@ -2665,7 +2746,7 @@
         <v>5</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="G10" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D10,G$4&lt;=$E10),1,0)</f>
@@ -2727,7 +2808,7 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="30"/>
       <c r="B11" s="31" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C11" s="30" t="n">
         <v>0</v>
@@ -2741,7 +2822,7 @@
         <v>5</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G11" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D11,G$4&lt;=$E11),1,0)</f>
@@ -2805,7 +2886,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -2819,7 +2900,7 @@
         <v>8</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="G12" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D12,G$4&lt;=$E12),1,0)</f>
@@ -2881,7 +2962,7 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30"/>
       <c r="B13" s="31" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C13" s="30" t="n">
         <v>0</v>
@@ -2895,7 +2976,7 @@
         <v>8</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G13" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D13,G$4&lt;=$E13),1,0)</f>
@@ -2959,7 +3040,7 @@
         <v>6</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>2</v>
@@ -2973,7 +3054,7 @@
         <v>10</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G14" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D14,G$4&lt;=$E14),1,0)</f>
@@ -3037,7 +3118,7 @@
         <v>7</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>1</v>
@@ -3051,7 +3132,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="G15" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D15,G$4&lt;=$E15),1,0)</f>
@@ -3115,7 +3196,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>2</v>
@@ -3129,7 +3210,7 @@
         <v>13</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G16" s="29" t="n">
         <f aca="false">IF(AND(G$4&gt;=$D16,G$4&lt;=$E16),1,0)</f>
@@ -3190,32 +3271,32 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="20" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C20" s="32"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C21" s="33"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D22" s="2" t="n">
         <f aca="false">SUM(C6:C16)-C8</f>
@@ -3224,7 +3305,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -3255,7 +3336,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -3265,386 +3346,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="34" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="35" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="35" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="35" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="35" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="35" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C9" s="36" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="35" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="35" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="35" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="35" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="35" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C14" s="36" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="35" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="35" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C16" s="36" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="35" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="35" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C18" s="36" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="35" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="B19" s="35" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="35" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="B20" s="35" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C20" s="36" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="35" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C21" s="36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="35" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C22" s="36" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="35" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B23" s="35" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C23" s="36" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="35" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B24" s="35" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="35" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B25" s="35" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C25" s="36" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="35" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B26" s="35" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C26" s="36" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="35" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B27" s="35" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C27" s="36" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="35" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B28" s="35" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="C28" s="36" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="35" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B29" s="35" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C29" s="36" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="35" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B30" s="35" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C30" s="36" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="35" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B31" s="35" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C31" s="36" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="35" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B32" s="35" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C32" s="36" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="35" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B33" s="35" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C33" s="36" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="35" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B34" s="35" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C34" s="36" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="35" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B35" s="35" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C35" s="36" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="35" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B36" s="35" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C36" s="36" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="35" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B37" s="35" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C37" s="36" t="s">
-        <v>229</v>
+        <v>230</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="35" t="s">
+        <v>226</v>
+      </c>
+      <c r="B38" s="35" t="s">
+        <v>231</v>
+      </c>
+      <c r="C38" s="36" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="35" t="s">
+        <v>233</v>
+      </c>
+      <c r="B39" s="35" t="s">
+        <v>234</v>
+      </c>
+      <c r="C39" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="35" t="s">
+        <v>233</v>
+      </c>
+      <c r="B40" s="35" t="s">
+        <v>236</v>
+      </c>
+      <c r="C40" s="36" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="35" t="s">
+        <v>233</v>
+      </c>
+      <c r="B41" s="35" t="s">
+        <v>238</v>
+      </c>
+      <c r="C41" s="36" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="35" t="s">
+        <v>233</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>240</v>
+      </c>
+      <c r="C42" s="36" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="35" t="s">
+        <v>242</v>
+      </c>
+      <c r="B43" s="35" t="s">
+        <v>243</v>
+      </c>
+      <c r="C43" s="36" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="35" t="s">
+        <v>242</v>
+      </c>
+      <c r="B44" s="35" t="s">
+        <v>245</v>
+      </c>
+      <c r="C44" s="36" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="35" t="s">
+        <v>247</v>
+      </c>
+      <c r="B45" s="35" t="s">
+        <v>248</v>
+      </c>
+      <c r="C45" s="36" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="35" t="s">
+        <v>247</v>
+      </c>
+      <c r="B46" s="35" t="s">
+        <v>250</v>
+      </c>
+      <c r="C46" s="36" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="35" t="s">
+        <v>247</v>
+      </c>
+      <c r="B47" s="35" t="s">
+        <v>252</v>
+      </c>
+      <c r="C47" s="36" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="35" t="s">
+        <v>254</v>
+      </c>
+      <c r="B48" s="35" t="s">
+        <v>255</v>
+      </c>
+      <c r="C48" s="36" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -3655,33 +3857,44 @@
     <hyperlink ref="C8" r:id="rId4" display="https://www.motor1.com/news/763606/amg-gt-xx-concept-first-look/"/>
     <hyperlink ref="C9" r:id="rId5" display="https://interestingengineering.com/photo-story/mercedes-amg-ev-concept-breaks-records"/>
     <hyperlink ref="C10" r:id="rId6" display="https://www.drivencarguide.co.nz/news/mercedes-amgs-concept-amg-gt-xx-packs-serious-tech-under-throwback-looks/"/>
-    <hyperlink ref="C11" r:id="rId7" display="https://www.mercedes-amg.com/en/gt-4-door-coupe"/>
-    <hyperlink ref="C12" r:id="rId8" display="https://group.mercedes-benz.com/company/production/news/axial-flux-motor-berlin.html"/>
-    <hyperlink ref="C13" r:id="rId9" display="https://www.electrive.com/2026/05/20/electric-powerhouse-mercedes-amg-unveils-gt-4-door-coupe/"/>
-    <hyperlink ref="C14" r:id="rId10" display="https://www.autocarindia.com/car-news/2026-mercedes-amg-gt-4-door-coupe-revealed-makes-up-to-1169hp-439771"/>
-    <hyperlink ref="C15" r:id="rId11" display="https://www.arenaev.com/mercedes_amg_gt_4_door_coup%c3%a9_gt_63_2026-specs-986.php"/>
-    <hyperlink ref="C16" r:id="rId12" display="https://www.automobile-catalog.com/car/2026/3653165/mercedes-amg_gt_63_4-door_coupe_ev.html"/>
-    <hyperlink ref="C17" r:id="rId13" display="https://newsroom.porsche.com/en/2024/products/porsche-the-new-taycan-turbo-gt-35479.html"/>
-    <hyperlink ref="C18" r:id="rId14" display="https://newsroom.porsche.com/dam/jcr:c96cbebc-3745-4700-b385-981a9c4fe91d/pag-taycan-turbo-gt-weissachpaket-td-en.pdf"/>
-    <hyperlink ref="C19" r:id="rId15" display="https://newsroom.porsche.com/en/2025/products/porsche-taycan-turbo-gt-most-powerful-poduction-porsche-38431.html"/>
-    <hyperlink ref="C20" r:id="rId16" display="https://www.audi.com/en/press-releases/audis-most-powerful-production-vehicle-the-new-rs-e-tron-gt-performance-16222"/>
-    <hyperlink ref="C21" r:id="rId17" display="https://uploads.audi-mediacenter.com/system/production/car_motorizations/1392/file_en/91bfc69ec55530e277b5023245b77c1c82772920/eTD-Audi-RS-e-tron-GT-performance-550kW_250515.pdf"/>
-    <hyperlink ref="C22" r:id="rId18" display="https://magazine.audi.com.au/article/peak-performance"/>
-    <hyperlink ref="C23" r:id="rId19" display="https://evkx.net/models/lotus/emeya/emeya_r/specifications"/>
-    <hyperlink ref="C24" r:id="rId20" display="https://data.carnewschina.com/database/lotus/lotus-emeya/2024"/>
-    <hyperlink ref="C25" r:id="rId21" display="https://evkx.net/models/tesla/model_s/model_s_plaid/specifications/"/>
-    <hyperlink ref="C26" r:id="rId22" display="https://lucidmotors.com/stories/final-production-specs-sapphire"/>
-    <hyperlink ref="C27" r:id="rId23" display="https://lucidmotors.com/media/document/lucid-air-sapphire-technical-specs-2024.pdf"/>
-    <hyperlink ref="C28" r:id="rId24" display="https://evkx.net/models/xiaomi/su7/su7_ultra/specifications"/>
-    <hyperlink ref="C29" r:id="rId25" display="https://carnewschina.com/2024/07/19/new-xiaomi-su7-ultra-with-1548-horsepower-and-v8s-motor-unveiled-in-china"/>
-    <hyperlink ref="C30" r:id="rId26" display="https://autotijd.be/en/specs/yangwang/u9/960-kw-awd-4586"/>
-    <hyperlink ref="C31" r:id="rId27" display="https://data.carnewschina.com/database/yangwang/yangwang-u9/2024/params"/>
-    <hyperlink ref="C32" r:id="rId28" display="https://www.cars24.com.au/car-news/yangwang-u9-track-edition-sets-global-ev-speed-record/"/>
-    <hyperlink ref="C33" r:id="rId29" display="https://web-cdn.rimac-automobili.com/wp-content/uploads/2023/11/20171226/Nevera_Technical-specifications.pdf"/>
-    <hyperlink ref="C34" r:id="rId30" display="https://www.rimac-automobili.com/nevera/"/>
-    <hyperlink ref="C35" r:id="rId31" display="https://www.maserati.com/us/en/models/granturismo/granturismo-folgore"/>
-    <hyperlink ref="C36" r:id="rId32" display="https://m.arenaev.com/maserati_granturismo_folgore_92kwh_2023-specs-amps-362.php"/>
-    <hyperlink ref="C37" r:id="rId33" display="https://unarte.org/wp-content/uploads/2026/08/Structura-anului-universitar-2026-2027.pdf"/>
+    <hyperlink ref="C11" r:id="rId7" display="https://media.mercedes-benz.com/en/article/dc62bb92-5082-42f1-bc9a-c838bc09e985"/>
+    <hyperlink ref="C12" r:id="rId8" display="https://media.mercedes-benz.com/en/article/b2d73049-f14b-4019-8da3-a0dd5e6dfb89"/>
+    <hyperlink ref="C13" r:id="rId9" display="https://media.mercedes-benz.com/en/article/c8b7109f-2287-4070-b776-9204da1513ef"/>
+    <hyperlink ref="C14" r:id="rId10" display="https://media.mercedes-benz.com/article/f037de81-64ba-4236-b555-75a5f4c3a56b"/>
+    <hyperlink ref="C15" r:id="rId11" display="https://media.mercedes-benz.com/en/article/bebac2af-acdc-465a-9538-adb0bf3d8ccf"/>
+    <hyperlink ref="C16" r:id="rId12" display="https://media.mercedes-benz.com/en/article/0955928c-b613-41b4-b754-08399bbfcccc"/>
+    <hyperlink ref="C17" r:id="rId13" display="https://www.mercedes-amg.com/en/gt-4-door-coupe"/>
+    <hyperlink ref="C18" r:id="rId14" display="https://group.mercedes-benz.com/company/production/news/axial-flux-motor-berlin.html"/>
+    <hyperlink ref="C19" r:id="rId15" display="https://www.electrive.com/2026/05/20/electric-powerhouse-mercedes-amg-unveils-gt-4-door-coupe/"/>
+    <hyperlink ref="C20" r:id="rId16" display="https://www.autocarindia.com/car-news/2026-mercedes-amg-gt-4-door-coupe-revealed-makes-up-to-1169hp-439771"/>
+    <hyperlink ref="C21" r:id="rId17" display="https://www.arenaev.com/mercedes_amg_gt_4_door_coup%c3%a9_gt_63_2026-specs-986.php"/>
+    <hyperlink ref="C22" r:id="rId18" display="https://www.automobile-catalog.com/car/2026/3653165/mercedes-amg_gt_63_4-door_coupe_ev.html"/>
+    <hyperlink ref="C23" r:id="rId19" display="https://newsroom.porsche.com/en/2024/products/porsche-the-new-taycan-turbo-gt-35479.html"/>
+    <hyperlink ref="C24" r:id="rId20" display="https://newsroom.porsche.com/dam/jcr:c96cbebc-3745-4700-b385-981a9c4fe91d/pag-taycan-turbo-gt-weissachpaket-td-en.pdf"/>
+    <hyperlink ref="C25" r:id="rId21" display="https://newsroom.porsche.com/en/2025/products/porsche-taycan-turbo-gt-most-powerful-poduction-porsche-38431.html"/>
+    <hyperlink ref="C26" r:id="rId22" display="https://www.audi.com/en/press-releases/audis-most-powerful-production-vehicle-the-new-rs-e-tron-gt-performance-16222"/>
+    <hyperlink ref="C27" r:id="rId23" display="https://uploads.audi-mediacenter.com/system/production/car_motorizations/1392/file_en/91bfc69ec55530e277b5023245b77c1c82772920/eTD-Audi-RS-e-tron-GT-performance-550kW_250515.pdf"/>
+    <hyperlink ref="C28" r:id="rId24" display="https://magazine.audi.com.au/article/peak-performance"/>
+    <hyperlink ref="C29" r:id="rId25" display="https://www.lotuscars.com/en/press/models/emeya"/>
+    <hyperlink ref="C30" r:id="rId26" display="https://www.lotuscars.com/en-GB/emeya/specifications"/>
+    <hyperlink ref="C31" r:id="rId27" display="https://evkx.net/models/lotus/emeya/emeya_r/specifications"/>
+    <hyperlink ref="C32" r:id="rId28" display="https://data.carnewschina.com/database/lotus/lotus-emeya/2024"/>
+    <hyperlink ref="C33" r:id="rId29" display="https://evkx.net/models/tesla/model_s/model_s_plaid/specifications/"/>
+    <hyperlink ref="C34" r:id="rId30" display="https://lucidmotors.com/stories/final-production-specs-sapphire"/>
+    <hyperlink ref="C35" r:id="rId31" display="https://lucidmotors.com/media/document/lucid-air-sapphire-technical-specs-2024.pdf"/>
+    <hyperlink ref="C36" r:id="rId32" display="https://evkx.net/models/xiaomi/su7/su7_ultra/specifications"/>
+    <hyperlink ref="C37" r:id="rId33" display="https://detail.zol.com.cn/2113/2112093/param.shtml"/>
+    <hyperlink ref="C38" r:id="rId34" display="https://carnewschina.com/2024/07/19/new-xiaomi-su7-ultra-with-1548-horsepower-and-v8s-motor-unveiled-in-china"/>
+    <hyperlink ref="C39" r:id="rId35" display="https://www.byd.com/us/news-list/YANGWANG-Launched-the-U9-Priced-at-1-68-Million-RMB"/>
+    <hyperlink ref="C40" r:id="rId36" display="https://autotijd.be/en/specs/yangwang/u9/960-kw-awd-4586"/>
+    <hyperlink ref="C41" r:id="rId37" display="https://data.carnewschina.com/database/yangwang/yangwang-u9/2024/params"/>
+    <hyperlink ref="C42" r:id="rId38" display="https://www.cars24.com.au/car-news/yangwang-u9-track-edition-sets-global-ev-speed-record/"/>
+    <hyperlink ref="C43" r:id="rId39" display="https://cloudfront.rimac-automobili.com/wp-content/uploads/2023/11/20171226/Nevera_Technical-specifications.pdf"/>
+    <hyperlink ref="C44" r:id="rId40" display="https://www.rimac-automobili.com/nevera/"/>
+    <hyperlink ref="C45" r:id="rId41" display="https://www.maserati.com/us/en/models/granturismo/granturismo-folgore"/>
+    <hyperlink ref="C46" r:id="rId42" display="https://www.media.stellantis.com/em-en/maserati/press/new-maserati-granturismo"/>
+    <hyperlink ref="C47" r:id="rId43" display="https://m.arenaev.com/maserati_granturismo_folgore_92kwh_2023-specs-amps-362.php"/>
+    <hyperlink ref="C48" r:id="rId44" display="https://unarte.org/wp-content/uploads/2026/08/Structura-anului-universitar-2026-2027.pdf"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>